<commit_message>
new analysis on h5
</commit_message>
<xml_diff>
--- a/case_studies/backbone/networks/existing/hydrogenPipelineOnshore.xlsx
+++ b/case_studies/backbone/networks/existing/hydrogenPipelineOnshore.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\backbone\networks\existing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E659AB-8ABA-4A19-9218-80FCB580DD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62266A4-1A3D-44D3-B5F4-D47DFEA21031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -935,22 +935,22 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -958,25 +958,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -984,25 +984,25 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1010,25 +1010,25 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1036,25 +1036,25 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1062,25 +1062,25 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1088,22 +1088,22 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="H8">
         <v>0</v>

</xml_diff>